<commit_message>
refactor: drop dead code and consolidate src/features into src/renderer/features
</commit_message>
<xml_diff>
--- a/examples/Inventory.xlsx
+++ b/examples/Inventory.xlsx
@@ -12,39 +12,42 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Stock</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Monitors</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>Laptops</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>Keyboards</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>tst</t>
+  </si>
   <si>
     <t>Item</t>
-  </si>
-  <si>
-    <t>Stock</t>
-  </si>
-  <si>
-    <t>Location</t>
-  </si>
-  <si>
-    <t>Monitors</t>
-  </si>
-  <si>
-    <t>A1</t>
-  </si>
-  <si>
-    <t>Laptops</t>
-  </si>
-  <si>
-    <t>A2</t>
-  </si>
-  <si>
-    <t>Keyboards</t>
-  </si>
-  <si>
-    <t>A3</t>
-  </si>
-  <si>
-    <t>123</t>
-  </si>
-  <si>
-    <t>tst</t>
   </si>
   <si>
     <t>Docking Stations</t>
@@ -442,7 +445,9 @@
   <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="5" width="10" customWidth="1"/>
+    <col min="1" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="14.428571428571429" customWidth="1"/>
+    <col min="4" max="100" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -494,9 +499,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>9</v>
+      </c>
+      <c r="E7" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="4:4" x14ac:dyDescent="0.25">
@@ -525,12 +533,12 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="3" width="10" customWidth="1"/>
+    <col min="1" max="100" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -541,35 +549,35 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2">
         <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3">
         <v>120</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B4">
         <v>200</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>